<commit_message>
Inicializar y limpiar Backend Legacy 2024 con README de instalación
</commit_message>
<xml_diff>
--- a/dssProject/Modelo_matemático/settings.xlsx
+++ b/dssProject/Modelo_matemático/settings.xlsx
@@ -2,34 +2,28 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$F$276</definedName>
-  </definedNames>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,33 +42,15 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -437,36 +413,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F276"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <dimension ref="A1:F273"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Máquina</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Bmax</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Proc</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>T. Proc</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
         <is>
           <t>Tclean</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
@@ -479,7 +455,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
@@ -505,7 +481,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
@@ -531,7 +507,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
@@ -553,14 +529,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>P_04</t>
+          <t>PR_01</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -572,18 +548,18 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Despalillado</t>
+          <t>Prensado</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PR_01</t>
+          <t>PR_02</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="C6" t="n">
         <v>7</v>
@@ -605,14 +581,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PR_02</t>
+          <t>PR_03</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -631,14 +607,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PR_03</t>
+          <t>PR_04</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="C8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -657,14 +633,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PR_04</t>
+          <t>PR_05</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="C9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -683,14 +659,14 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PR_05</t>
+          <t>PR_06</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -709,14 +685,14 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PR_06</t>
+          <t>PR_07</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
@@ -735,14 +711,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PR_07</t>
+          <t>PR_08</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
@@ -761,14 +737,14 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PR_08</t>
+          <t>PR_09</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C13" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -787,14 +763,14 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PR_09</t>
+          <t>PR_10</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
@@ -813,11 +789,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PR_10</t>
+          <t>PR_11</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C15" t="n">
         <v>7</v>
@@ -839,14 +815,14 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PR_11</t>
+          <t>PR_12</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C16" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
@@ -865,14 +841,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PR_12</t>
+          <t>CubaPF_01</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>80</v>
+        <v>100000</v>
       </c>
       <c r="C17" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -884,14 +860,14 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Prensado</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CubaPF_01</t>
+          <t>CubaPF_02</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -910,14 +886,14 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CubaPF_02</t>
+          <t>CubaPF_03</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -936,14 +912,14 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CubaPF_03</t>
+          <t>CubaPF_04</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -962,14 +938,14 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CubaPF_04</t>
+          <t>CubaPF_05</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -988,14 +964,14 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CubaPF_05</t>
+          <t>CubaPF_06</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1014,14 +990,14 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CubaPF_06</t>
+          <t>CubaPF_07</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1040,14 +1016,14 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CubaPF_07</t>
+          <t>CubaPF_08</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1066,14 +1042,14 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CubaPF_08</t>
+          <t>CubaPF_09</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1092,14 +1068,14 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CubaPF_09</t>
+          <t>CubaPF_10</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1118,14 +1094,14 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CubaPF_10</t>
+          <t>CubaPF_11</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1144,14 +1120,14 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CubaPF_11</t>
+          <t>CubaPF_12</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1170,14 +1146,14 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CubaPF_12</t>
+          <t>CubaPF_13</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1196,14 +1172,14 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CubaPF_13</t>
+          <t>CubaPF_14</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1222,14 +1198,14 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CubaPF_14</t>
+          <t>CubaPF_15</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1248,14 +1224,14 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CubaPF_15</t>
+          <t>CubaPF_16</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1274,18 +1250,18 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CubaPF_16</t>
+          <t>CubaPF_17</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>100000</v>
+        <v>50000</v>
       </c>
       <c r="C33" t="n">
         <v>1</v>
@@ -1300,14 +1276,14 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CubaPF_17</t>
+          <t>CubaPF_18</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1326,14 +1302,14 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CubaPF_18</t>
+          <t>CubaPF_19</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1352,14 +1328,14 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CubaPF_19</t>
+          <t>CubaPF_20</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1378,14 +1354,14 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CubaPF_20</t>
+          <t>CubaPF_21</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1404,14 +1380,14 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CubaPF_21</t>
+          <t>CubaPF_22</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1430,14 +1406,14 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CubaPF_22</t>
+          <t>CubaPF_23</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1456,14 +1432,14 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CubaPF_23</t>
+          <t>CubaPF_24</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1482,18 +1458,18 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Pre-flotacion</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CubaPF_24</t>
+          <t>FLT_01</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="C41" t="n">
         <v>1</v>
@@ -1508,21 +1484,21 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Pre-flotación</t>
+          <t>Flotacion</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>FLT_01</t>
+          <t>FLT_02</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>100000</v>
+        <v>60000</v>
       </c>
       <c r="C42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D42" t="n">
         <v>0</v>
@@ -1534,21 +1510,21 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Flotación</t>
+          <t>Flotacion</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>FLT_02</t>
+          <t>FLT_03</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>100000</v>
+        <v>60000</v>
       </c>
       <c r="C43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D43" t="n">
         <v>0</v>
@@ -1560,21 +1536,21 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Flotación</t>
+          <t>Flotacion</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>FLT_03</t>
+          <t>CubaF_01</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>100000</v>
+        <v>65000</v>
       </c>
       <c r="C44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D44" t="n">
         <v>0</v>
@@ -1586,21 +1562,21 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Flotación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>FLT_04</t>
+          <t>CubaF_02</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>100000</v>
+        <v>65000</v>
       </c>
       <c r="C45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D45" t="n">
         <v>0</v>
@@ -1612,14 +1588,14 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Flotación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CubaF_01</t>
+          <t>CubaF_03</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1638,14 +1614,14 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CubaF_02</t>
+          <t>CubaF_04</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1664,14 +1640,14 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CubaF_03</t>
+          <t>CubaF_05</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1690,14 +1666,14 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CubaF_04</t>
+          <t>CubaF_06</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1716,14 +1692,14 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CubaF_05</t>
+          <t>CubaF_07</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1742,14 +1718,14 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CubaF_06</t>
+          <t>CubaF_08</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1768,14 +1744,14 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CubaF_07</t>
+          <t>CubaF_09</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1794,14 +1770,14 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CubaF_08</t>
+          <t>CubaF_10</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1820,14 +1796,14 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CubaF_09</t>
+          <t>CubaF_11</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1846,14 +1822,14 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CubaF_10</t>
+          <t>CubaF_12</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1872,14 +1848,14 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CubaF_11</t>
+          <t>CubaF_13</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1898,14 +1874,14 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CubaF_12</t>
+          <t>CubaF_14</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1924,14 +1900,14 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CubaF_13</t>
+          <t>CubaF_15</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1950,14 +1926,14 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CubaF_14</t>
+          <t>CubaF_16</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1976,14 +1952,14 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CubaF_15</t>
+          <t>CubaF_17</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -2002,14 +1978,14 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CubaF_16</t>
+          <t>CubaF_18</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -2028,14 +2004,14 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CubaF_17</t>
+          <t>CubaF_19</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -2054,14 +2030,14 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CubaF_18</t>
+          <t>CubaF_20</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -2080,14 +2056,14 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CubaF_19</t>
+          <t>CubaF_21</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -2106,14 +2082,14 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CubaF_20</t>
+          <t>CubaF_22</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -2132,14 +2108,14 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CubaF_21</t>
+          <t>CubaF_23</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -2158,14 +2134,14 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CubaF_22</t>
+          <t>CubaF_24</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -2184,14 +2160,14 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CubaF_23</t>
+          <t>CubaF_25</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -2210,14 +2186,14 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CubaF_24</t>
+          <t>CubaF_26</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -2236,14 +2212,14 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CubaF_25</t>
+          <t>CubaF_27</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -2262,14 +2238,14 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CubaF_26</t>
+          <t>CubaF_28</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -2288,14 +2264,14 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CubaF_27</t>
+          <t>CubaF_29</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -2314,14 +2290,14 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CubaF_28</t>
+          <t>CubaF_30</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -2340,14 +2316,14 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CubaF_29</t>
+          <t>CubaF_31</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -2366,14 +2342,14 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CubaF_30</t>
+          <t>CubaF_32</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -2392,14 +2368,14 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CubaF_31</t>
+          <t>CubaF_33</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -2418,14 +2394,14 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CubaF_32</t>
+          <t>CubaF_34</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -2444,14 +2420,14 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CubaF_33</t>
+          <t>CubaF_35</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -2470,14 +2446,14 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CubaF_34</t>
+          <t>CubaF_36</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -2496,14 +2472,14 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CubaF_35</t>
+          <t>CubaF_37</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -2522,14 +2498,14 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CubaF_36</t>
+          <t>CubaF_38</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -2548,14 +2524,14 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CubaF_37</t>
+          <t>CubaF_39</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -2574,14 +2550,14 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CubaF_38</t>
+          <t>CubaF_40</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -2600,14 +2576,14 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CubaF_39</t>
+          <t>CubaF_41</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -2626,14 +2602,14 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CubaF_40</t>
+          <t>CubaF_42</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -2652,14 +2628,14 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CubaF_41</t>
+          <t>CubaF_43</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -2678,14 +2654,14 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CubaF_42</t>
+          <t>CubaF_44</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -2704,14 +2680,14 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CubaF_43</t>
+          <t>CubaF_45</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -2730,14 +2706,14 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CubaF_44</t>
+          <t>CubaF_46</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -2756,14 +2732,14 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CubaF_45</t>
+          <t>CubaF_47</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -2782,14 +2758,14 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CubaF_46</t>
+          <t>CubaF_48</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -2808,14 +2784,14 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CubaF_47</t>
+          <t>CubaF_49</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -2834,14 +2810,14 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CubaF_48</t>
+          <t>CubaF_50</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -2860,14 +2836,14 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CubaF_49</t>
+          <t>CubaF_51</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -2886,14 +2862,14 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CubaF_50</t>
+          <t>CubaF_52</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -2912,14 +2888,14 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CubaF_51</t>
+          <t>CubaF_53</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -2938,14 +2914,14 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CubaF_52</t>
+          <t>CubaF_54</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -2964,14 +2940,14 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CubaF_53</t>
+          <t>CubaF_55</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -2990,14 +2966,14 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CubaF_54</t>
+          <t>CubaF_56</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -3016,14 +2992,14 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CubaF_55</t>
+          <t>CubaF_57</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -3042,14 +3018,14 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CubaF_56</t>
+          <t>CubaF_58</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -3068,14 +3044,14 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>CubaF_57</t>
+          <t>CubaF_59</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -3094,14 +3070,14 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>CubaF_58</t>
+          <t>CubaF_60</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -3120,14 +3096,14 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>CubaF_59</t>
+          <t>CubaF_61</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -3146,14 +3122,14 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>CubaF_60</t>
+          <t>CubaF_62</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -3172,14 +3148,14 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>CubaF_61</t>
+          <t>CubaF_63</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -3198,14 +3174,14 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>CubaF_62</t>
+          <t>CubaF_64</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -3224,14 +3200,14 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>CubaF_63</t>
+          <t>CubaF_65</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -3250,14 +3226,14 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>CubaF_64</t>
+          <t>CubaF_66</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -3276,14 +3252,14 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>CubaF_65</t>
+          <t>CubaF_67</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -3302,14 +3278,14 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>CubaF_66</t>
+          <t>CubaF_68</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -3328,14 +3304,14 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>CubaF_67</t>
+          <t>CubaF_69</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -3354,14 +3330,14 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>CubaF_68</t>
+          <t>CubaF_70</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -3380,14 +3356,14 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>CubaF_69</t>
+          <t>CubaF_71</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -3406,14 +3382,14 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>CubaF_70</t>
+          <t>CubaF_72</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -3432,14 +3408,14 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>CubaF_71</t>
+          <t>CubaF_73</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -3458,14 +3434,14 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>CubaF_72</t>
+          <t>CubaF_74</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -3484,14 +3460,14 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>CubaF_73</t>
+          <t>CubaF_75</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -3510,14 +3486,14 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>CubaF_74</t>
+          <t>CubaF_76</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -3536,14 +3512,14 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>CubaF_75</t>
+          <t>CubaF_77</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -3562,14 +3538,14 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>CubaF_76</t>
+          <t>CubaF_78</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -3588,14 +3564,14 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>CubaF_77</t>
+          <t>CubaF_79</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -3614,14 +3590,14 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>CubaF_78</t>
+          <t>CubaF_80</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -3640,14 +3616,14 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>CubaF_79</t>
+          <t>CubaF_81</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -3666,14 +3642,14 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>CubaF_80</t>
+          <t>CubaF_82</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -3692,14 +3668,14 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>CubaF_81</t>
+          <t>CubaF_83</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -3718,14 +3694,14 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>CubaF_82</t>
+          <t>CubaF_84</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -3744,14 +3720,14 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>CubaF_83</t>
+          <t>CubaF_85</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -3770,14 +3746,14 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>CubaF_84</t>
+          <t>CubaF_86</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -3796,14 +3772,14 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>CubaF_85</t>
+          <t>CubaF_87</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -3822,14 +3798,14 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>CubaF_86</t>
+          <t>CubaF_88</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -3848,14 +3824,14 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>CubaF_87</t>
+          <t>CubaF_89</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -3874,14 +3850,14 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>CubaF_88</t>
+          <t>CubaF_90</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -3900,14 +3876,14 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>CubaF_89</t>
+          <t>CubaF_91</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -3926,14 +3902,14 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>CubaF_90</t>
+          <t>CubaF_92</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -3952,14 +3928,14 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>CubaF_91</t>
+          <t>CubaF_93</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -3978,14 +3954,14 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>CubaF_92</t>
+          <t>CubaF_94</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -4004,14 +3980,14 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>CubaF_93</t>
+          <t>CubaF_95</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -4030,14 +4006,14 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>CubaF_94</t>
+          <t>CubaF_96</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -4056,14 +4032,14 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>CubaF_95</t>
+          <t>CubaF_97</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -4082,14 +4058,14 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>CubaF_96</t>
+          <t>CubaF_98</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -4108,14 +4084,14 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>CubaF_97</t>
+          <t>CubaF_99</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -4134,14 +4110,14 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>CubaF_98</t>
+          <t>CubaF_100</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -4160,14 +4136,14 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>CubaF_99</t>
+          <t>CubaF_101</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -4186,14 +4162,14 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>CubaF_100</t>
+          <t>CubaF_102</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -4212,14 +4188,14 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>CubaF_101</t>
+          <t>CubaF_103</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -4238,14 +4214,14 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>CubaF_102</t>
+          <t>CubaF_104</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -4264,14 +4240,14 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>CubaF_103</t>
+          <t>CubaF_105</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -4290,14 +4266,14 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>CubaF_104</t>
+          <t>CubaF_106</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -4316,14 +4292,14 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>CubaF_105</t>
+          <t>CubaF_107</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -4342,14 +4318,14 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>CubaF_106</t>
+          <t>CubaF_108</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -4368,14 +4344,14 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>CubaF_107</t>
+          <t>CubaF_109</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -4394,14 +4370,14 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>CubaF_108</t>
+          <t>CubaF_110</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -4420,14 +4396,14 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>CubaF_109</t>
+          <t>CubaF_111</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -4446,14 +4422,14 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>CubaF_110</t>
+          <t>CubaF_112</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -4472,14 +4448,14 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>CubaF_111</t>
+          <t>CubaF_113</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -4498,14 +4474,14 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>CubaF_112</t>
+          <t>CubaF_114</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -4524,14 +4500,14 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>CubaF_113</t>
+          <t>CubaF_115</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -4550,14 +4526,14 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>CubaF_114</t>
+          <t>CubaF_116</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -4576,14 +4552,14 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>CubaF_115</t>
+          <t>CubaF_117</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -4602,14 +4578,14 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>CubaF_116</t>
+          <t>CubaF_118</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -4628,14 +4604,14 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>CubaF_117</t>
+          <t>CubaF_119</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -4654,14 +4630,14 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>CubaF_118</t>
+          <t>CubaF_120</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -4680,14 +4656,14 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>CubaF_119</t>
+          <t>CubaF_121</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -4706,14 +4682,14 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>CubaF_120</t>
+          <t>CubaF_122</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -4732,14 +4708,14 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>CubaF_121</t>
+          <t>CubaF_123</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -4758,14 +4734,14 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>CubaF_122</t>
+          <t>CubaF_124</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -4784,14 +4760,14 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>CubaF_123</t>
+          <t>CubaF_125</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -4810,14 +4786,14 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>CubaF_124</t>
+          <t>CubaF_126</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -4836,14 +4812,14 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>CubaF_125</t>
+          <t>CubaF_127</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -4862,14 +4838,14 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>CubaF_126</t>
+          <t>CubaF_128</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -4888,14 +4864,14 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>CubaF_127</t>
+          <t>CubaF_129</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -4914,14 +4890,14 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>CubaF_128</t>
+          <t>CubaF_130</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -4940,14 +4916,14 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>CubaF_129</t>
+          <t>CubaF_131</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -4966,14 +4942,14 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>CubaF_130</t>
+          <t>CubaF_132</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -4992,14 +4968,14 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>CubaF_131</t>
+          <t>CubaF_133</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -5018,14 +4994,14 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>CubaF_132</t>
+          <t>CubaF_134</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -5044,14 +5020,14 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>CubaF_133</t>
+          <t>CubaF_135</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -5070,14 +5046,14 @@
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>CubaF_134</t>
+          <t>CubaF_136</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -5096,14 +5072,14 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>CubaF_135</t>
+          <t>CubaF_137</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -5122,14 +5098,14 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>CubaF_136</t>
+          <t>CubaF_138</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -5148,14 +5124,14 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>CubaF_137</t>
+          <t>CubaF_139</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -5174,14 +5150,14 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>CubaF_138</t>
+          <t>CubaF_140</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -5200,14 +5176,14 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>CubaF_139</t>
+          <t>CubaF_141</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -5226,14 +5202,14 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>CubaF_140</t>
+          <t>CubaF_142</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -5252,14 +5228,14 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>CubaF_141</t>
+          <t>CubaF_143</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -5278,14 +5254,14 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>CubaF_142</t>
+          <t>CubaF_144</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -5304,14 +5280,14 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>CubaF_143</t>
+          <t>CubaF_145</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -5330,14 +5306,14 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>CubaF_144</t>
+          <t>CubaF_146</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -5356,14 +5332,14 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>CubaF_145</t>
+          <t>CubaF_147</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -5382,14 +5358,14 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>CubaF_146</t>
+          <t>CubaF_148</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -5408,14 +5384,14 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>CubaF_147</t>
+          <t>CubaF_149</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -5434,14 +5410,14 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>CubaF_148</t>
+          <t>CubaF_150</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -5460,14 +5436,14 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>CubaF_149</t>
+          <t>CubaF_151</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -5486,14 +5462,14 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>CubaF_150</t>
+          <t>CubaF_152</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -5512,14 +5488,14 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>CubaF_151</t>
+          <t>CubaF_153</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -5538,14 +5514,14 @@
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>CubaF_152</t>
+          <t>CubaF_154</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -5564,14 +5540,14 @@
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>CubaF_153</t>
+          <t>CubaF_155</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -5590,14 +5566,14 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>CubaF_154</t>
+          <t>CubaF_156</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -5616,14 +5592,14 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>CubaF_155</t>
+          <t>CubaF_157</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -5642,14 +5618,14 @@
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>CubaF_156</t>
+          <t>CubaF_158</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -5668,14 +5644,14 @@
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>CubaF_157</t>
+          <t>CubaF_159</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -5694,14 +5670,14 @@
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>CubaF_158</t>
+          <t>CubaF_160</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -5720,14 +5696,14 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>CubaF_159</t>
+          <t>CubaF_161</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -5746,14 +5722,14 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>CubaF_160</t>
+          <t>CubaF_162</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -5772,14 +5748,14 @@
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>CubaF_161</t>
+          <t>CubaF_163</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -5798,14 +5774,14 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>CubaF_162</t>
+          <t>CubaF_164</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -5824,14 +5800,14 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>CubaF_163</t>
+          <t>CubaF_165</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -5850,14 +5826,14 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>CubaF_164</t>
+          <t>CubaF_166</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -5876,14 +5852,14 @@
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>CubaF_165</t>
+          <t>CubaF_167</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -5902,14 +5878,14 @@
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>CubaF_166</t>
+          <t>CubaF_168</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -5928,14 +5904,14 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>CubaF_167</t>
+          <t>CubaF_169</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -5954,14 +5930,14 @@
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>CubaF_168</t>
+          <t>CubaF_170</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -5980,14 +5956,14 @@
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>CubaF_169</t>
+          <t>CubaF_171</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -6006,14 +5982,14 @@
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>CubaF_170</t>
+          <t>CubaF_172</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -6032,14 +6008,14 @@
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>CubaF_171</t>
+          <t>CubaF_173</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -6058,14 +6034,14 @@
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>CubaF_172</t>
+          <t>CubaF_174</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -6084,14 +6060,14 @@
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>CubaF_173</t>
+          <t>CubaF_175</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -6110,14 +6086,14 @@
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>CubaF_174</t>
+          <t>CubaF_176</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -6136,14 +6112,14 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>CubaF_175</t>
+          <t>CubaF_177</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -6162,14 +6138,14 @@
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>CubaF_176</t>
+          <t>CubaF_178</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -6188,14 +6164,14 @@
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>CubaF_177</t>
+          <t>CubaF_179</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -6214,14 +6190,14 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>CubaF_178</t>
+          <t>CubaF_180</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -6240,14 +6216,14 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>CubaF_179</t>
+          <t>CubaF_181</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -6266,14 +6242,14 @@
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>CubaF_180</t>
+          <t>CubaF_182</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -6292,14 +6268,14 @@
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>CubaF_181</t>
+          <t>CubaF_183</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -6318,14 +6294,14 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>CubaF_182</t>
+          <t>CubaF_184</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -6344,14 +6320,14 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>CubaF_183</t>
+          <t>CubaF_185</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -6370,14 +6346,14 @@
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>CubaF_184</t>
+          <t>CubaF_186</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -6396,14 +6372,14 @@
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>CubaF_185</t>
+          <t>CubaF_187</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -6422,14 +6398,14 @@
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>CubaF_186</t>
+          <t>CubaF_188</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -6448,14 +6424,14 @@
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>CubaF_187</t>
+          <t>CubaF_189</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -6474,14 +6450,14 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>CubaF_188</t>
+          <t>CubaF_190</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -6500,14 +6476,14 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>CubaF_189</t>
+          <t>CubaF_191</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -6526,14 +6502,14 @@
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>CubaF_190</t>
+          <t>CubaF_192</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -6552,14 +6528,14 @@
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>CubaF_191</t>
+          <t>CubaF_193</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -6578,14 +6554,14 @@
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>CubaF_192</t>
+          <t>CubaF_194</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -6604,14 +6580,14 @@
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>CubaF_193</t>
+          <t>CubaF_195</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -6630,14 +6606,14 @@
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>CubaF_194</t>
+          <t>CubaF_196</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -6656,14 +6632,14 @@
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>CubaF_195</t>
+          <t>CubaF_197</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -6682,14 +6658,14 @@
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>CubaF_196</t>
+          <t>CubaF_198</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -6708,14 +6684,14 @@
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>CubaF_197</t>
+          <t>CubaF_199</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -6734,14 +6710,14 @@
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>CubaF_198</t>
+          <t>CubaF_200</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -6760,14 +6736,14 @@
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>CubaF_199</t>
+          <t>CubaF_201</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -6786,14 +6762,14 @@
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>CubaF_200</t>
+          <t>CubaF_202</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -6812,14 +6788,14 @@
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>CubaF_201</t>
+          <t>CubaF_203</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -6838,14 +6814,14 @@
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>CubaF_202</t>
+          <t>CubaF_204</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -6864,14 +6840,14 @@
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>CubaF_203</t>
+          <t>CubaF_205</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -6890,14 +6866,14 @@
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>CubaF_204</t>
+          <t>CubaF_206</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -6916,14 +6892,14 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>CubaF_205</t>
+          <t>CubaF_207</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -6942,14 +6918,14 @@
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>CubaF_206</t>
+          <t>CubaF_208</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -6968,14 +6944,14 @@
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>CubaF_207</t>
+          <t>CubaF_209</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -6994,14 +6970,14 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>CubaF_208</t>
+          <t>CubaF_210</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -7020,14 +6996,14 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>CubaF_209</t>
+          <t>CubaF_211</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -7046,14 +7022,14 @@
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>CubaF_210</t>
+          <t>CubaF_212</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -7072,14 +7048,14 @@
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>CubaF_211</t>
+          <t>CubaF_213</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -7098,14 +7074,14 @@
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>CubaF_212</t>
+          <t>CubaF_214</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -7124,14 +7100,14 @@
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>CubaF_213</t>
+          <t>CubaF_215</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -7150,14 +7126,14 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>CubaF_214</t>
+          <t>CubaF_216</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -7176,14 +7152,14 @@
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>CubaF_215</t>
+          <t>CubaF_217</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -7202,14 +7178,14 @@
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>CubaF_216</t>
+          <t>CubaF_218</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -7228,14 +7204,14 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>CubaF_217</t>
+          <t>CubaF_219</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -7254,14 +7230,14 @@
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>CubaF_218</t>
+          <t>CubaF_220</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -7280,14 +7256,14 @@
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>CubaF_219</t>
+          <t>CubaF_221</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -7306,14 +7282,14 @@
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>CubaF_220</t>
+          <t>CubaF_222</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -7332,14 +7308,14 @@
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>CubaF_221</t>
+          <t>CubaF_223</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -7358,14 +7334,14 @@
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>CubaF_222</t>
+          <t>CubaF_224</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -7384,14 +7360,14 @@
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>CubaF_223</t>
+          <t>CubaF_225</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -7410,14 +7386,14 @@
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>CubaF_224</t>
+          <t>CubaF_226</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -7436,14 +7412,14 @@
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>CubaF_225</t>
+          <t>CubaF_227</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -7462,14 +7438,14 @@
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>CubaF_226</t>
+          <t>CubaF_228</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -7488,14 +7464,14 @@
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>CubaF_227</t>
+          <t>CubaF_229</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -7514,14 +7490,14 @@
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>Fermentación</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>CubaF_228</t>
+          <t>CubaF_230</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -7540,90 +7516,11 @@
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>Fermentación</t>
-        </is>
-      </c>
-    </row>
-    <row r="274">
-      <c r="A274" t="inlineStr">
-        <is>
-          <t>CubaF_229</t>
-        </is>
-      </c>
-      <c r="B274" t="n">
-        <v>65000</v>
-      </c>
-      <c r="C274" t="n">
-        <v>1</v>
-      </c>
-      <c r="D274" t="n">
-        <v>0</v>
-      </c>
-      <c r="E274" t="inlineStr">
-        <is>
-          <t>Habilitado</t>
-        </is>
-      </c>
-      <c r="F274" t="inlineStr">
-        <is>
-          <t>Fermentación</t>
-        </is>
-      </c>
-    </row>
-    <row r="275">
-      <c r="A275" t="inlineStr">
-        <is>
-          <t>CubaF_230</t>
-        </is>
-      </c>
-      <c r="B275" t="n">
-        <v>65000</v>
-      </c>
-      <c r="C275" t="n">
-        <v>1</v>
-      </c>
-      <c r="D275" t="n">
-        <v>0</v>
-      </c>
-      <c r="E275" t="inlineStr">
-        <is>
-          <t>Habilitado</t>
-        </is>
-      </c>
-      <c r="F275" t="inlineStr">
-        <is>
-          <t>Fermentación</t>
-        </is>
-      </c>
-    </row>
-    <row r="276">
-      <c r="A276" t="inlineStr">
-        <is>
-          <t>P_05</t>
-        </is>
-      </c>
-      <c r="B276" t="n">
-        <v>100</v>
-      </c>
-      <c r="C276" t="n">
-        <v>1</v>
-      </c>
-      <c r="D276" t="n">
-        <v>0</v>
-      </c>
-      <c r="E276" t="inlineStr">
-        <is>
-          <t>Habilitado</t>
-        </is>
-      </c>
-      <c r="F276" t="inlineStr">
-        <is>
-          <t>Despalillado</t>
+          <t>Fermentacion</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F276"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>